<commit_message>
contract status inquiry - Inprogress
</commit_message>
<xml_diff>
--- a/src/data/update-unit.xlsx
+++ b/src/data/update-unit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright Workspace\github_workspaces\Sakani_Playwright\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F120CF07-D0D0-45E0-8203-43C2C73CBECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{468D884F-B978-44B7-BBE4-AFC6CBCE7D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -845,10 +845,10 @@
     <t>financial_subsidized</t>
   </si>
   <si>
-    <t>beneficiary, non_bene, company</t>
-  </si>
-  <si>
-    <t>partners</t>
+    <t>web, mobile, partners, third_party, ops_team</t>
+  </si>
+  <si>
+    <t>beneficiary</t>
   </si>
 </sst>
 </file>
@@ -1623,26 +1623,26 @@
         <v>40</v>
       </c>
       <c r="W2" s="2"/>
-      <c r="X2" s="6">
-        <v>66000</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>66000</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>66000</v>
+      <c r="X2" s="3">
+        <v>100000</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>100000</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>100000</v>
       </c>
       <c r="AA2" s="6">
         <v>150</v>
       </c>
-      <c r="AB2" s="6">
-        <v>66000</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>66000</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>66000</v>
+      <c r="AB2" s="3">
+        <v>100000</v>
+      </c>
+      <c r="AC2" s="3">
+        <v>100000</v>
+      </c>
+      <c r="AD2" s="3">
+        <v>100000</v>
       </c>
       <c r="AE2" s="6">
         <v>3</v>
@@ -1716,10 +1716,10 @@
         <v>75</v>
       </c>
       <c r="BL2" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="BM2" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="BM2" s="5" t="s">
-        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>